<commit_message>
Actualizacion los botones de  frmconexion
</commit_message>
<xml_diff>
--- a/ReporteGasolina/Documentos/GASOLINA CARGA INICIAL.xlsx
+++ b/ReporteGasolina/Documentos/GASOLINA CARGA INICIAL.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Terceros\fortia\Senosiain\Reporte Gasolina\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Desarrollos\DesarrollosVisual\ReporteGasolina\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B624EC1-5CF4-48E0-AE4B-AE5D1C54BF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{406C9A8B-7AFA-4BBC-945C-BAFFC80C3970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{737309C1-BAA0-413D-AC0B-3F32CFE088C5}"/>
   </bookViews>

</xml_diff>

<commit_message>
Actualizacion Repositorios al 02-sep-2026
</commit_message>
<xml_diff>
--- a/ReporteGasolina/Documentos/GASOLINA CARGA INICIAL.xlsx
+++ b/ReporteGasolina/Documentos/GASOLINA CARGA INICIAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Desarrollos\DesarrollosVisual\ReporteGasolina\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CAABDD0-1E72-4C89-BA6C-6FBF93F82265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7320AE03-4511-4072-8B7A-1F2C83CB7D38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{737309C1-BAA0-413D-AC0B-3F32CFE088C5}"/>
   </bookViews>
@@ -225,7 +225,7 @@
     <t>ZAPOPAN</t>
   </si>
   <si>
-    <t>Agosto</t>
+    <t>octubre</t>
   </si>
 </sst>
 </file>
@@ -657,7 +657,7 @@
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="6"/>
       <c r="B4" s="8">
-        <v>2026</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -665,6 +665,9 @@
         <v>3</v>
       </c>
       <c r="B5" s="2">
+        <v>8.7000000000000011</v>
+      </c>
+      <c r="E5" s="2">
         <v>21.75</v>
       </c>
     </row>
@@ -673,8 +676,9 @@
         <v>4</v>
       </c>
       <c r="B6" s="2">
-        <v>0</v>
-      </c>
+        <v>8.1760000000000002</v>
+      </c>
+      <c r="D6" s="2"/>
       <c r="E6" s="2">
         <v>20.440000000000001</v>
       </c>
@@ -684,6 +688,9 @@
         <v>5</v>
       </c>
       <c r="B7" s="2">
+        <v>8.9320000000000004</v>
+      </c>
+      <c r="E7" s="2">
         <v>22.33</v>
       </c>
     </row>
@@ -692,6 +699,9 @@
         <v>6</v>
       </c>
       <c r="B8" s="2">
+        <v>6.5400000000000009</v>
+      </c>
+      <c r="E8" s="2">
         <v>16.350000000000001</v>
       </c>
     </row>
@@ -700,6 +710,9 @@
         <v>7</v>
       </c>
       <c r="B9" s="2">
+        <v>8.548</v>
+      </c>
+      <c r="E9" s="2">
         <v>21.37</v>
       </c>
     </row>
@@ -708,6 +721,9 @@
         <v>8</v>
       </c>
       <c r="B10" s="2">
+        <v>7.9120000000000008</v>
+      </c>
+      <c r="E10" s="2">
         <v>19.78</v>
       </c>
     </row>
@@ -716,6 +732,9 @@
         <v>9</v>
       </c>
       <c r="B11" s="2">
+        <v>8.3800000000000008</v>
+      </c>
+      <c r="E11" s="2">
         <v>20.95</v>
       </c>
     </row>
@@ -724,6 +743,9 @@
         <v>10</v>
       </c>
       <c r="B12" s="3">
+        <v>8.32</v>
+      </c>
+      <c r="E12" s="3">
         <v>20.8</v>
       </c>
     </row>
@@ -732,6 +754,9 @@
         <v>11</v>
       </c>
       <c r="B13" s="2">
+        <v>8.26</v>
+      </c>
+      <c r="E13" s="2">
         <v>20.65</v>
       </c>
     </row>
@@ -740,6 +765,9 @@
         <v>12</v>
       </c>
       <c r="B14" s="2">
+        <v>9.1720000000000006</v>
+      </c>
+      <c r="E14" s="2">
         <v>22.93</v>
       </c>
     </row>
@@ -748,6 +776,9 @@
         <v>13</v>
       </c>
       <c r="B15" s="2">
+        <v>7.944</v>
+      </c>
+      <c r="E15" s="2">
         <v>19.86</v>
       </c>
     </row>
@@ -756,390 +787,537 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
+        <v>8.4920000000000009</v>
+      </c>
+      <c r="E16" s="2">
         <v>21.23</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B17" s="2">
+        <v>8.016</v>
+      </c>
+      <c r="E17" s="2">
         <v>20.04</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="2">
+        <v>8.1</v>
+      </c>
+      <c r="E18" s="2">
         <v>20.25</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B19" s="2">
+        <v>8.2240000000000002</v>
+      </c>
+      <c r="E19" s="2">
         <v>20.56</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B20" s="2">
+        <v>8.5080000000000009</v>
+      </c>
+      <c r="E20" s="2">
         <v>21.27</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B21" s="2">
+        <v>8.4440000000000008</v>
+      </c>
+      <c r="E21" s="2">
         <v>21.11</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="2">
+        <v>8.14</v>
+      </c>
+      <c r="E22" s="2">
         <v>20.350000000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="2">
+        <v>8.4280000000000008</v>
+      </c>
+      <c r="E23" s="2">
         <v>21.07</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B24" s="2">
+        <v>8.4920000000000009</v>
+      </c>
+      <c r="E24" s="2">
         <v>21.23</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B25" s="2">
+        <v>8.58</v>
+      </c>
+      <c r="E25" s="2">
         <v>21.45</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B26" s="2">
+        <v>8.4440000000000008</v>
+      </c>
+      <c r="E26" s="2">
         <v>21.11</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B27" s="2">
+        <v>8.620000000000001</v>
+      </c>
+      <c r="E27" s="2">
         <v>21.55</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B28" s="2">
+        <v>8.2760000000000016</v>
+      </c>
+      <c r="E28" s="2">
         <v>20.69</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B29" s="2">
+        <v>9.0680000000000014</v>
+      </c>
+      <c r="E29" s="2">
         <v>22.67</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B30" s="2">
+        <v>6.5360000000000005</v>
+      </c>
+      <c r="E30" s="2">
         <v>16.34</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="2">
+        <v>8.4680000000000017</v>
+      </c>
+      <c r="E31" s="2">
         <v>21.17</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B32" s="2">
+        <v>8.452</v>
+      </c>
+      <c r="E32" s="2">
         <v>21.13</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B33" s="2">
+        <v>7.8680000000000012</v>
+      </c>
+      <c r="E33" s="2">
         <v>19.670000000000002</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B34" s="2">
+        <v>8.7439999999999998</v>
+      </c>
+      <c r="E34" s="2">
         <v>21.86</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B35" s="2">
+        <v>8.2319999999999993</v>
+      </c>
+      <c r="E35" s="2">
         <v>20.58</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B36" s="2">
+        <v>8.6880000000000006</v>
+      </c>
+      <c r="E36" s="2">
         <v>21.72</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B37" s="2">
+        <v>6.8520000000000003</v>
+      </c>
+      <c r="E37" s="2">
         <v>17.13</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
         <v>36</v>
       </c>
       <c r="B38" s="2">
+        <v>6.3640000000000008</v>
+      </c>
+      <c r="E38" s="2">
         <v>15.91</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B39" s="2">
+        <v>8.7520000000000007</v>
+      </c>
+      <c r="E39" s="2">
         <v>21.88</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B40" s="2">
+        <v>7.9640000000000004</v>
+      </c>
+      <c r="E40" s="2">
         <v>19.91</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B41" s="2">
+        <v>8.3559999999999999</v>
+      </c>
+      <c r="E41" s="2">
         <v>20.89</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B42" s="2">
+        <v>8.0200000000000014</v>
+      </c>
+      <c r="E42" s="2">
         <v>20.05</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B43" s="2">
+        <v>8.4280000000000008</v>
+      </c>
+      <c r="E43" s="2">
         <v>21.07</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B44" s="2">
+        <v>8.072000000000001</v>
+      </c>
+      <c r="E44" s="2">
         <v>20.18</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B45" s="9">
+        <v>6.88</v>
+      </c>
+      <c r="E45" s="9">
         <v>17.2</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B46" s="2">
+        <v>8.1760000000000002</v>
+      </c>
+      <c r="E46" s="2">
         <v>20.440000000000001</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B47" s="2">
+        <v>8.3400000000000016</v>
+      </c>
+      <c r="E47" s="2">
         <v>20.85</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B48" s="2">
+        <v>7.024</v>
+      </c>
+      <c r="E48" s="2">
         <v>17.559999999999999</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B49" s="2">
+        <v>7.8920000000000003</v>
+      </c>
+      <c r="E49" s="2">
         <v>19.73</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B50" s="2">
+        <v>8.1840000000000011</v>
+      </c>
+      <c r="E50" s="2">
         <v>20.46</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
       <c r="B51" s="2">
+        <v>8.6080000000000005</v>
+      </c>
+      <c r="E51" s="2">
         <v>21.52</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B52" s="3">
+        <v>8.0400000000000009</v>
+      </c>
+      <c r="E52" s="3">
         <v>20.100000000000001</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B53" s="2">
+        <v>8.4280000000000008</v>
+      </c>
+      <c r="E53" s="2">
         <v>21.07</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B54" s="2">
+        <v>8.0280000000000005</v>
+      </c>
+      <c r="E54" s="2">
         <v>20.07</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B55" s="2">
+        <v>8.4280000000000008</v>
+      </c>
+      <c r="E55" s="2">
         <v>21.07</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B56" s="2">
+        <v>8.2520000000000007</v>
+      </c>
+      <c r="E56" s="2">
         <v>20.63</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B57" s="2">
+        <v>8.2240000000000002</v>
+      </c>
+      <c r="E57" s="2">
         <v>20.56</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B58" s="2">
+        <v>8.3079999999999998</v>
+      </c>
+      <c r="E58" s="2">
         <v>20.77</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B59" s="2">
+        <v>7.9720000000000004</v>
+      </c>
+      <c r="E59" s="2">
         <v>19.93</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B60" s="2">
+        <v>8.2919999999999998</v>
+      </c>
+      <c r="E60" s="2">
         <v>20.73</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B61" s="2">
+        <v>8.4440000000000008</v>
+      </c>
+      <c r="E61" s="2">
         <v>21.11</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>60</v>
       </c>
       <c r="B62" s="2">
+        <v>8.1480000000000015</v>
+      </c>
+      <c r="E62" s="2">
         <v>20.37</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B63" s="2">
+        <v>8.5960000000000001</v>
+      </c>
+      <c r="E63" s="2">
         <v>21.49</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B64" s="2">
+        <v>21.07</v>
+      </c>
+      <c r="E64" s="2">
         <v>21.07</v>
       </c>
     </row>

</xml_diff>